<commit_message>
Vision: trained-model classifier, training toolchain, deep sleep
- vision/training: Python 3.12 venv toolchain (sort_photos, train,
  quantize, smoke_test). MobileNetV2 transfer learning -> int8 .espdl via
  ESP-PPQ; equalization off + TQT on (smoke test: int8 67% -> 100%)
- classify_model.cpp: ESP-DL loads /sdcard/model.espdl if present, else
  the blob classifier runs; deploy/rollback is one file on the SD card
- vision.c: results.csv log per photo; reference photos saved as known
  "none" examples
- Deep sleep: MSG_SLEEP over the link; P4 sleeps after finishing its
  current job and wakes on its UART RX line (EXT1, ANY_LOW). Main board
  sends MSG_SLEEP before its own sleep and a wake PING at boot
- link.c: typed inbox; jobs admitted by a counting semaphore (ERR_BUSY
  when one is in flight), control messages never refused
- Parts list updates

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CrowBox_PartsList.xlsx
+++ b/CrowBox_PartsList.xlsx
@@ -9747,8 +9747,10 @@
       <c r="J1" s="16" t="s">
         <v>631</v>
       </c>
-      <c r="K1" s="16" t="s">
-        <v>632</v>
+      <c r="K1" s="16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Have? (Y = received, O = ordered)</t>
+        </is>
       </c>
       <c r="L1" s="16" t="s">
         <v>15</v>
@@ -9797,9 +9799,13 @@
         <f aca="false">H2*I2</f>
         <v>133.8</v>
       </c>
-      <c r="K2" s="27"/>
+      <c r="K2" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L2" s="26" t="n">
-        <f aca="false">IF(UPPER(K2)="Y",0,J2)</f>
+        <f aca="false">IF(OR(UPPER(K2)="Y",UPPER(K2)="O"),0,J2)</f>
         <v>133.8</v>
       </c>
       <c r="M2" s="5" t="s">
@@ -9845,9 +9851,13 @@
         <f aca="false">H3*I3</f>
         <v>44</v>
       </c>
-      <c r="K3" s="27"/>
+      <c r="K3" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L3" s="26" t="n">
-        <f aca="false">IF(UPPER(K3)="Y",0,J3)</f>
+        <f aca="false">IF(OR(UPPER(K3)="Y",UPPER(K3)="O"),0,J3)</f>
         <v>44</v>
       </c>
       <c r="M3" s="5" t="s">
@@ -9894,9 +9904,13 @@
         <f aca="false">H4*I4</f>
         <v>18</v>
       </c>
-      <c r="K4" s="27"/>
+      <c r="K4" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L4" s="26" t="n">
-        <f aca="false">IF(UPPER(K4)="Y",0,J4)</f>
+        <f aca="false">IF(OR(UPPER(K4)="Y",UPPER(K4)="O"),0,J4)</f>
         <v>18</v>
       </c>
       <c r="M4" s="5" t="s">
@@ -9943,9 +9957,13 @@
         <f aca="false">H5*I5</f>
         <v>7</v>
       </c>
-      <c r="K5" s="27"/>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L5" s="26" t="n">
-        <f aca="false">IF(UPPER(K5)="Y",0,J5)</f>
+        <f aca="false">IF(OR(UPPER(K5)="Y",UPPER(K5)="O"),0,J5)</f>
         <v>7</v>
       </c>
       <c r="M5" s="5" t="s">
@@ -9992,9 +10010,13 @@
         <f aca="false">H6*I6</f>
         <v>7</v>
       </c>
-      <c r="K6" s="27"/>
+      <c r="K6" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L6" s="26" t="n">
-        <f aca="false">IF(UPPER(K6)="Y",0,J6)</f>
+        <f aca="false">IF(OR(UPPER(K6)="Y",UPPER(K6)="O"),0,J6)</f>
         <v>7</v>
       </c>
       <c r="M6" s="5" t="s">
@@ -10041,9 +10063,13 @@
         <f aca="false">H7*I7</f>
         <v>11</v>
       </c>
-      <c r="K7" s="27"/>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L7" s="26" t="n">
-        <f aca="false">IF(UPPER(K7)="Y",0,J7)</f>
+        <f aca="false">IF(OR(UPPER(K7)="Y",UPPER(K7)="O"),0,J7)</f>
         <v>11</v>
       </c>
       <c r="M7" s="5" t="s">
@@ -10090,9 +10116,13 @@
         <f aca="false">H8*I8</f>
         <v>8</v>
       </c>
-      <c r="K8" s="27"/>
+      <c r="K8" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L8" s="26" t="n">
-        <f aca="false">IF(UPPER(K8)="Y",0,J8)</f>
+        <f aca="false">IF(OR(UPPER(K8)="Y",UPPER(K8)="O"),0,J8)</f>
         <v>8</v>
       </c>
       <c r="M8" s="5" t="s">
@@ -10139,9 +10169,13 @@
         <f aca="false">H9*I9</f>
         <v>6</v>
       </c>
-      <c r="K9" s="27"/>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L9" s="26" t="n">
-        <f aca="false">IF(UPPER(K9)="Y",0,J9)</f>
+        <f aca="false">IF(OR(UPPER(K9)="Y",UPPER(K9)="O"),0,J9)</f>
         <v>6</v>
       </c>
       <c r="M9" s="5" t="s">
@@ -10188,9 +10222,13 @@
         <f aca="false">H10*I10</f>
         <v>8</v>
       </c>
-      <c r="K10" s="27"/>
+      <c r="K10" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L10" s="26" t="n">
-        <f aca="false">IF(UPPER(K10)="Y",0,J10)</f>
+        <f aca="false">IF(OR(UPPER(K10)="Y",UPPER(K10)="O"),0,J10)</f>
         <v>8</v>
       </c>
       <c r="M10" s="5" t="s">
@@ -10237,9 +10275,13 @@
         <f aca="false">H11*I11</f>
         <v>10</v>
       </c>
-      <c r="K11" s="27"/>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L11" s="26" t="n">
-        <f aca="false">IF(UPPER(K11)="Y",0,J11)</f>
+        <f aca="false">IF(OR(UPPER(K11)="Y",UPPER(K11)="O"),0,J11)</f>
         <v>10</v>
       </c>
       <c r="M11" s="5" t="s">
@@ -10288,7 +10330,7 @@
       </c>
       <c r="K12" s="27"/>
       <c r="L12" s="26" t="n">
-        <f aca="false">IF(UPPER(K12)="Y",0,J12)</f>
+        <f aca="false">IF(OR(UPPER(K12)="Y",UPPER(K12)="O"),0,J12)</f>
         <v>8</v>
       </c>
       <c r="M12" s="5" t="s">
@@ -10335,9 +10377,13 @@
         <f aca="false">H13*I13</f>
         <v>8</v>
       </c>
-      <c r="K13" s="27"/>
+      <c r="K13" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L13" s="26" t="n">
-        <f aca="false">IF(UPPER(K13)="Y",0,J13)</f>
+        <f aca="false">IF(OR(UPPER(K13)="Y",UPPER(K13)="O"),0,J13)</f>
         <v>8</v>
       </c>
       <c r="M13" s="5" t="s">
@@ -10384,9 +10430,13 @@
         <f aca="false">H14*I14</f>
         <v>6</v>
       </c>
-      <c r="K14" s="27"/>
+      <c r="K14" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L14" s="26" t="n">
-        <f aca="false">IF(UPPER(K14)="Y",0,J14)</f>
+        <f aca="false">IF(OR(UPPER(K14)="Y",UPPER(K14)="O"),0,J14)</f>
         <v>6</v>
       </c>
       <c r="M14" s="5" t="s">
@@ -10433,9 +10483,13 @@
         <f aca="false">H15*I15</f>
         <v>5</v>
       </c>
-      <c r="K15" s="27"/>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L15" s="26" t="n">
-        <f aca="false">IF(UPPER(K15)="Y",0,J15)</f>
+        <f aca="false">IF(OR(UPPER(K15)="Y",UPPER(K15)="O"),0,J15)</f>
         <v>5</v>
       </c>
       <c r="M15" s="5" t="s">
@@ -10482,9 +10536,13 @@
         <f aca="false">H16*I16</f>
         <v>4</v>
       </c>
-      <c r="K16" s="27"/>
+      <c r="K16" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L16" s="26" t="n">
-        <f aca="false">IF(UPPER(K16)="Y",0,J16)</f>
+        <f aca="false">IF(OR(UPPER(K16)="Y",UPPER(K16)="O"),0,J16)</f>
         <v>4</v>
       </c>
       <c r="M16" s="5" t="s">
@@ -10511,8 +10569,7 @@
         <v>697</v>
       </c>
       <c r="E17" s="14" t="n">
-        <f aca="false">SUMIF(Fasteners!$A$2:$A$41,"M5 spacer 5mm",Fasteners!$C$2:$C$41)</f>
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="F17" s="5" t="s">
         <v>650</v>
@@ -10533,7 +10590,7 @@
       </c>
       <c r="K17" s="27"/>
       <c r="L17" s="26" t="n">
-        <f aca="false">IF(UPPER(K17)="Y",0,J17)</f>
+        <f aca="false">IF(OR(UPPER(K17)="Y",UPPER(K17)="O"),0,J17)</f>
         <v>8</v>
       </c>
       <c r="M17" s="5" t="s">
@@ -10542,8 +10599,10 @@
       <c r="N17" s="5" t="s">
         <v>698</v>
       </c>
-      <c r="O17" s="5" t="s">
-        <v>652</v>
+      <c r="O17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DROPPED: front panel standoffs are stacks of 5 M5 washers instead.</t>
+        </is>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10580,9 +10639,13 @@
         <f aca="false">H18*I18</f>
         <v>5</v>
       </c>
-      <c r="K18" s="27"/>
+      <c r="K18" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L18" s="26" t="n">
-        <f aca="false">IF(UPPER(K18)="Y",0,J18)</f>
+        <f aca="false">IF(OR(UPPER(K18)="Y",UPPER(K18)="O"),0,J18)</f>
         <v>5</v>
       </c>
       <c r="M18" s="5" t="s">
@@ -10629,9 +10692,13 @@
         <f aca="false">H19*I19</f>
         <v>5</v>
       </c>
-      <c r="K19" s="27"/>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L19" s="26" t="n">
-        <f aca="false">IF(UPPER(K19)="Y",0,J19)</f>
+        <f aca="false">IF(OR(UPPER(K19)="Y",UPPER(K19)="O"),0,J19)</f>
         <v>5</v>
       </c>
       <c r="M19" s="5" t="s">
@@ -10678,9 +10745,13 @@
         <f aca="false">H20*I20</f>
         <v>4</v>
       </c>
-      <c r="K20" s="27"/>
+      <c r="K20" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L20" s="26" t="n">
-        <f aca="false">IF(UPPER(K20)="Y",0,J20)</f>
+        <f aca="false">IF(OR(UPPER(K20)="Y",UPPER(K20)="O"),0,J20)</f>
         <v>4</v>
       </c>
       <c r="M20" s="5" t="s">
@@ -10727,9 +10798,13 @@
         <f aca="false">H21*I21</f>
         <v>4</v>
       </c>
-      <c r="K21" s="27"/>
+      <c r="K21" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L21" s="26" t="n">
-        <f aca="false">IF(UPPER(K21)="Y",0,J21)</f>
+        <f aca="false">IF(OR(UPPER(K21)="Y",UPPER(K21)="O"),0,J21)</f>
         <v>4</v>
       </c>
       <c r="M21" s="5" t="s">
@@ -10756,8 +10831,7 @@
         <v>713</v>
       </c>
       <c r="E22" s="14" t="n">
-        <f aca="false">SUMIF(Fasteners!$A$2:$A$41,"Spacer M4x11",Fasteners!$C$2:$C$41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F22" s="5" t="s">
         <v>650</v>
@@ -10778,7 +10852,7 @@
       </c>
       <c r="K22" s="27"/>
       <c r="L22" s="26" t="n">
-        <f aca="false">IF(UPPER(K22)="Y",0,J22)</f>
+        <f aca="false">IF(OR(UPPER(K22)="Y",UPPER(K22)="O"),0,J22)</f>
         <v>5</v>
       </c>
       <c r="M22" s="5" t="s">
@@ -10787,8 +10861,10 @@
       <c r="N22" s="5" t="s">
         <v>714</v>
       </c>
-      <c r="O22" s="5" t="s">
-        <v>715</v>
+      <c r="O22" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DROPPED: load cell spacer is 3 M4 hex nuts + 3 M4 washers instead.</t>
+        </is>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10805,8 +10881,7 @@
         <v>718</v>
       </c>
       <c r="E23" s="14" t="n">
-        <f aca="false">SUMIF(Fasteners!$A$2:$A$41,"Spacer M4x5",Fasteners!$C$2:$C$41)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23" s="5" t="s">
         <v>650</v>
@@ -10827,7 +10902,7 @@
       </c>
       <c r="K23" s="27"/>
       <c r="L23" s="26" t="n">
-        <f aca="false">IF(UPPER(K23)="Y",0,J23)</f>
+        <f aca="false">IF(OR(UPPER(K23)="Y",UPPER(K23)="O"),0,J23)</f>
         <v>4</v>
       </c>
       <c r="M23" s="5" t="s">
@@ -10836,8 +10911,10 @@
       <c r="N23" s="5" t="s">
         <v>719</v>
       </c>
-      <c r="O23" s="5" t="s">
-        <v>715</v>
+      <c r="O23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DROPPED: load cell spacer is 6 M4 washers instead.</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10876,7 +10953,7 @@
       </c>
       <c r="K24" s="27"/>
       <c r="L24" s="26" t="n">
-        <f aca="false">IF(UPPER(K24)="Y",0,J24)</f>
+        <f aca="false">IF(OR(UPPER(K24)="Y",UPPER(K24)="O"),0,J24)</f>
         <v>8</v>
       </c>
       <c r="M24" s="5" t="s">
@@ -10925,7 +11002,7 @@
       </c>
       <c r="K25" s="27"/>
       <c r="L25" s="26" t="n">
-        <f aca="false">IF(UPPER(K25)="Y",0,J25)</f>
+        <f aca="false">IF(OR(UPPER(K25)="Y",UPPER(K25)="O"),0,J25)</f>
         <v>6</v>
       </c>
       <c r="M25" s="5" t="s">
@@ -10974,7 +11051,7 @@
       </c>
       <c r="K26" s="27"/>
       <c r="L26" s="26" t="n">
-        <f aca="false">IF(UPPER(K26)="Y",0,J26)</f>
+        <f aca="false">IF(OR(UPPER(K26)="Y",UPPER(K26)="O"),0,J26)</f>
         <v>5</v>
       </c>
       <c r="M26" s="5" t="s">
@@ -11021,7 +11098,7 @@
       </c>
       <c r="K27" s="27"/>
       <c r="L27" s="26" t="n">
-        <f aca="false">IF(UPPER(K27)="Y",0,J27)</f>
+        <f aca="false">IF(OR(UPPER(K27)="Y",UPPER(K27)="O"),0,J27)</f>
         <v>4</v>
       </c>
       <c r="M27" s="5" t="s">
@@ -11067,9 +11144,13 @@
         <f aca="false">H28*I28</f>
         <v>12</v>
       </c>
-      <c r="K28" s="27"/>
+      <c r="K28" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L28" s="26" t="n">
-        <f aca="false">IF(UPPER(K28)="Y",0,J28)</f>
+        <f aca="false">IF(OR(UPPER(K28)="Y",UPPER(K28)="O"),0,J28)</f>
         <v>12</v>
       </c>
       <c r="M28" s="5" t="s">
@@ -11119,7 +11200,7 @@
       </c>
       <c r="K29" s="27"/>
       <c r="L29" s="26" t="n">
-        <f aca="false">IF(UPPER(K29)="Y",0,J29)</f>
+        <f aca="false">IF(OR(UPPER(K29)="Y",UPPER(K29)="O"),0,J29)</f>
         <v>8</v>
       </c>
       <c r="M29" s="5" t="s">
@@ -11167,7 +11248,7 @@
       </c>
       <c r="K30" s="27"/>
       <c r="L30" s="26" t="n">
-        <f aca="false">IF(UPPER(K30)="Y",0,J30)</f>
+        <f aca="false">IF(OR(UPPER(K30)="Y",UPPER(K30)="O"),0,J30)</f>
         <v>10</v>
       </c>
       <c r="M30" s="5" t="s">
@@ -11215,7 +11296,7 @@
       </c>
       <c r="K31" s="27"/>
       <c r="L31" s="26" t="n">
-        <f aca="false">IF(UPPER(K31)="Y",0,J31)</f>
+        <f aca="false">IF(OR(UPPER(K31)="Y",UPPER(K31)="O"),0,J31)</f>
         <v>42</v>
       </c>
       <c r="M31" s="5" t="s">
@@ -11261,7 +11342,7 @@
       </c>
       <c r="K32" s="27"/>
       <c r="L32" s="26" t="n">
-        <f aca="false">IF(UPPER(K32)="Y",0,J32)</f>
+        <f aca="false">IF(OR(UPPER(K32)="Y",UPPER(K32)="O"),0,J32)</f>
         <v>17</v>
       </c>
       <c r="M32" s="5" t="s">
@@ -11307,7 +11388,7 @@
       </c>
       <c r="K33" s="27"/>
       <c r="L33" s="26" t="n">
-        <f aca="false">IF(UPPER(K33)="Y",0,J33)</f>
+        <f aca="false">IF(OR(UPPER(K33)="Y",UPPER(K33)="O"),0,J33)</f>
         <v>9</v>
       </c>
       <c r="M33" s="5" t="s">
@@ -11355,7 +11436,7 @@
       </c>
       <c r="K34" s="27"/>
       <c r="L34" s="26" t="n">
-        <f aca="false">IF(UPPER(K34)="Y",0,J34)</f>
+        <f aca="false">IF(OR(UPPER(K34)="Y",UPPER(K34)="O"),0,J34)</f>
         <v>18</v>
       </c>
       <c r="M34" s="5" t="s">
@@ -11403,7 +11484,7 @@
       </c>
       <c r="K35" s="27"/>
       <c r="L35" s="26" t="n">
-        <f aca="false">IF(UPPER(K35)="Y",0,J35)</f>
+        <f aca="false">IF(OR(UPPER(K35)="Y",UPPER(K35)="O"),0,J35)</f>
         <v>3</v>
       </c>
       <c r="M35" s="5" t="s">
@@ -11449,7 +11530,7 @@
       </c>
       <c r="K36" s="27"/>
       <c r="L36" s="26" t="n">
-        <f aca="false">IF(UPPER(K36)="Y",0,J36)</f>
+        <f aca="false">IF(OR(UPPER(K36)="Y",UPPER(K36)="O"),0,J36)</f>
         <v>3</v>
       </c>
       <c r="M36" s="5" t="s">
@@ -11497,7 +11578,7 @@
       </c>
       <c r="K37" s="27"/>
       <c r="L37" s="26" t="n">
-        <f aca="false">IF(UPPER(K37)="Y",0,J37)</f>
+        <f aca="false">IF(OR(UPPER(K37)="Y",UPPER(K37)="O"),0,J37)</f>
         <v>12</v>
       </c>
       <c r="M37" s="5" t="s">
@@ -11545,7 +11626,7 @@
       </c>
       <c r="K38" s="27"/>
       <c r="L38" s="26" t="n">
-        <f aca="false">IF(UPPER(K38)="Y",0,J38)</f>
+        <f aca="false">IF(OR(UPPER(K38)="Y",UPPER(K38)="O"),0,J38)</f>
         <v>20</v>
       </c>
       <c r="M38" s="5" t="s">
@@ -11593,7 +11674,7 @@
       </c>
       <c r="K39" s="27"/>
       <c r="L39" s="26" t="n">
-        <f aca="false">IF(UPPER(K39)="Y",0,J39)</f>
+        <f aca="false">IF(OR(UPPER(K39)="Y",UPPER(K39)="O"),0,J39)</f>
         <v>40</v>
       </c>
       <c r="M39" s="5" t="s">
@@ -11641,7 +11722,7 @@
       </c>
       <c r="K40" s="27"/>
       <c r="L40" s="26" t="n">
-        <f aca="false">IF(UPPER(K40)="Y",0,J40)</f>
+        <f aca="false">IF(OR(UPPER(K40)="Y",UPPER(K40)="O"),0,J40)</f>
         <v>32</v>
       </c>
       <c r="M40" s="5" t="s">
@@ -11689,7 +11770,7 @@
       </c>
       <c r="K41" s="27"/>
       <c r="L41" s="26" t="n">
-        <f aca="false">IF(UPPER(K41)="Y",0,J41)</f>
+        <f aca="false">IF(OR(UPPER(K41)="Y",UPPER(K41)="O"),0,J41)</f>
         <v>22</v>
       </c>
       <c r="M41" s="5" t="s">
@@ -11737,7 +11818,7 @@
       </c>
       <c r="K42" s="27"/>
       <c r="L42" s="26" t="n">
-        <f aca="false">IF(UPPER(K42)="Y",0,J42)</f>
+        <f aca="false">IF(OR(UPPER(K42)="Y",UPPER(K42)="O"),0,J42)</f>
         <v>160</v>
       </c>
       <c r="M42" s="5" t="s">
@@ -11783,9 +11864,13 @@
         <f aca="false">H43*I43</f>
         <v>28</v>
       </c>
-      <c r="K43" s="27"/>
+      <c r="K43" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L43" s="26" t="n">
-        <f aca="false">IF(UPPER(K43)="Y",0,J43)</f>
+        <f aca="false">IF(OR(UPPER(K43)="Y",UPPER(K43)="O"),0,J43)</f>
         <v>28</v>
       </c>
       <c r="M43" s="5" t="s">
@@ -11837,7 +11922,7 @@
         </is>
       </c>
       <c r="L44" s="26" t="n">
-        <f aca="false">IF(UPPER(K44)="Y",0,J44)</f>
+        <f aca="false">IF(OR(UPPER(K44)="Y",UPPER(K44)="O"),0,J44)</f>
         <v>8</v>
       </c>
       <c r="M44" s="5" t="s">
@@ -11887,9 +11972,13 @@
         <f aca="false">H45*I45</f>
         <v>8</v>
       </c>
-      <c r="K45" s="27"/>
+      <c r="K45" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L45" s="26" t="n">
-        <f aca="false">IF(UPPER(K45)="Y",0,J45)</f>
+        <f aca="false">IF(OR(UPPER(K45)="Y",UPPER(K45)="O"),0,J45)</f>
         <v>8</v>
       </c>
       <c r="M45" s="5" t="s">
@@ -11937,7 +12026,7 @@
         </is>
       </c>
       <c r="L46" s="26" t="n">
-        <f aca="false">IF(UPPER(K46)="Y",0,J46)</f>
+        <f aca="false">IF(OR(UPPER(K46)="Y",UPPER(K46)="O"),0,J46)</f>
         <v>5</v>
       </c>
       <c r="M46" s="5" t="s">
@@ -11989,7 +12078,7 @@
         </is>
       </c>
       <c r="L47" s="26" t="n">
-        <f aca="false">IF(UPPER(K47)="Y",0,J47)</f>
+        <f aca="false">IF(OR(UPPER(K47)="Y",UPPER(K47)="O"),0,J47)</f>
         <v>5</v>
       </c>
       <c r="M47" s="5" t="s">
@@ -12035,9 +12124,13 @@
         <f aca="false">H48*I48</f>
         <v>9</v>
       </c>
-      <c r="K48" s="27"/>
+      <c r="K48" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L48" s="26" t="n">
-        <f aca="false">IF(UPPER(K48)="Y",0,J48)</f>
+        <f aca="false">IF(OR(UPPER(K48)="Y",UPPER(K48)="O"),0,J48)</f>
         <v>9</v>
       </c>
       <c r="M48" s="5" t="s">
@@ -12089,7 +12182,7 @@
         </is>
       </c>
       <c r="L49" s="26" t="n">
-        <f aca="false">IF(UPPER(K49)="Y",0,J49)</f>
+        <f aca="false">IF(OR(UPPER(K49)="Y",UPPER(K49)="O"),0,J49)</f>
         <v>6</v>
       </c>
       <c r="M49" s="5" t="s">
@@ -12135,9 +12228,13 @@
         <f aca="false">H50*I50</f>
         <v>10</v>
       </c>
-      <c r="K50" s="27"/>
+      <c r="K50" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L50" s="26" t="n">
-        <f aca="false">IF(UPPER(K50)="Y",0,J50)</f>
+        <f aca="false">IF(OR(UPPER(K50)="Y",UPPER(K50)="O"),0,J50)</f>
         <v>10</v>
       </c>
       <c r="M50" s="5" t="s">
@@ -12181,9 +12278,13 @@
         <f aca="false">H51*I51</f>
         <v>15</v>
       </c>
-      <c r="K51" s="27"/>
+      <c r="K51" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L51" s="26" t="n">
-        <f aca="false">IF(UPPER(K51)="Y",0,J51)</f>
+        <f aca="false">IF(OR(UPPER(K51)="Y",UPPER(K51)="O"),0,J51)</f>
         <v>15</v>
       </c>
       <c r="M51" s="5" t="s">
@@ -12233,7 +12334,7 @@
         </is>
       </c>
       <c r="L52" s="26" t="n">
-        <f aca="false">IF(UPPER(K52)="Y",0,J52)</f>
+        <f aca="false">IF(OR(UPPER(K52)="Y",UPPER(K52)="O"),0,J52)</f>
         <v>7</v>
       </c>
       <c r="M52" s="5" t="s">
@@ -12285,7 +12386,7 @@
         </is>
       </c>
       <c r="L53" s="26" t="n">
-        <f aca="false">IF(UPPER(K53)="Y",0,J53)</f>
+        <f aca="false">IF(OR(UPPER(K53)="Y",UPPER(K53)="O"),0,J53)</f>
         <v>6</v>
       </c>
       <c r="M53" s="5" t="s">
@@ -12335,7 +12436,7 @@
         </is>
       </c>
       <c r="L54" s="26" t="n">
-        <f aca="false">IF(UPPER(K54)="Y",0,J54)</f>
+        <f aca="false">IF(OR(UPPER(K54)="Y",UPPER(K54)="O"),0,J54)</f>
         <v>4</v>
       </c>
       <c r="M54" s="5" t="s">
@@ -12381,9 +12482,13 @@
         <f aca="false">H55*I55</f>
         <v>7</v>
       </c>
-      <c r="K55" s="27"/>
+      <c r="K55" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Y</t>
+        </is>
+      </c>
       <c r="L55" s="26" t="n">
-        <f aca="false">IF(UPPER(K55)="Y",0,J55)</f>
+        <f aca="false">IF(OR(UPPER(K55)="Y",UPPER(K55)="O"),0,J55)</f>
         <v>7</v>
       </c>
       <c r="M55" s="5" t="s">
@@ -12435,7 +12540,7 @@
         </is>
       </c>
       <c r="L56" s="26" t="n">
-        <f aca="false">IF(UPPER(K56)="Y",0,J56)</f>
+        <f aca="false">IF(OR(UPPER(K56)="Y",UPPER(K56)="O"),0,J56)</f>
         <v>8</v>
       </c>
       <c r="M56" s="5" t="s">
@@ -12483,7 +12588,7 @@
       </c>
       <c r="K57" s="27"/>
       <c r="L57" s="26" t="n">
-        <f aca="false">IF(UPPER(K57)="Y",0,J57)</f>
+        <f aca="false">IF(OR(UPPER(K57)="Y",UPPER(K57)="O"),0,J57)</f>
         <v>7</v>
       </c>
       <c r="M57" s="5" t="s">
@@ -12531,7 +12636,7 @@
       </c>
       <c r="K58" s="27"/>
       <c r="L58" s="26" t="n">
-        <f aca="false">IF(UPPER(K58)="Y",0,J58)</f>
+        <f aca="false">IF(OR(UPPER(K58)="Y",UPPER(K58)="O"),0,J58)</f>
         <v>7</v>
       </c>
       <c r="M58" s="5" t="s">
@@ -12577,9 +12682,13 @@
         <f aca="false">H59*I59</f>
         <v>25</v>
       </c>
-      <c r="K59" s="27"/>
+      <c r="K59" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L59" s="26" t="n">
-        <f aca="false">IF(UPPER(K59)="Y",0,J59)</f>
+        <f aca="false">IF(OR(UPPER(K59)="Y",UPPER(K59)="O"),0,J59)</f>
         <v>25</v>
       </c>
       <c r="M59" s="5" t="s">
@@ -12627,9 +12736,13 @@
         <f aca="false">H60*I60</f>
         <v>49</v>
       </c>
-      <c r="K60" s="27"/>
+      <c r="K60" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L60" s="26" t="n">
-        <f aca="false">IF(UPPER(K60)="Y",0,J60)</f>
+        <f aca="false">IF(OR(UPPER(K60)="Y",UPPER(K60)="O"),0,J60)</f>
         <v>49</v>
       </c>
       <c r="M60" s="5" t="s">
@@ -12677,9 +12790,13 @@
         <f aca="false">H61*I61</f>
         <v>12</v>
       </c>
-      <c r="K61" s="27"/>
+      <c r="K61" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L61" s="26" t="n">
-        <f aca="false">IF(UPPER(K61)="Y",0,J61)</f>
+        <f aca="false">IF(OR(UPPER(K61)="Y",UPPER(K61)="O"),0,J61)</f>
         <v>12</v>
       </c>
       <c r="M61" s="5" t="s">
@@ -12729,9 +12846,13 @@
         <f aca="false">H62*I62</f>
         <v>20</v>
       </c>
-      <c r="K62" s="27"/>
+      <c r="K62" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L62" s="26" t="n">
-        <f aca="false">IF(UPPER(K62)="Y",0,J62)</f>
+        <f aca="false">IF(OR(UPPER(K62)="Y",UPPER(K62)="O"),0,J62)</f>
         <v>20</v>
       </c>
       <c r="M62" s="5" t="s">
@@ -12785,9 +12906,13 @@
         <f aca="false">H63*I63</f>
         <v>25</v>
       </c>
-      <c r="K63" s="27"/>
+      <c r="K63" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L63" s="26" t="n">
-        <f aca="false">IF(UPPER(K63)="Y",0,J63)</f>
+        <f aca="false">IF(OR(UPPER(K63)="Y",UPPER(K63)="O"),0,J63)</f>
         <v>25</v>
       </c>
       <c r="M63" s="5" t="s">
@@ -12837,7 +12962,7 @@
       </c>
       <c r="K64" s="27"/>
       <c r="L64" s="26" t="n">
-        <f aca="false">IF(UPPER(K64)="Y",0,J64)</f>
+        <f aca="false">IF(OR(UPPER(K64)="Y",UPPER(K64)="O"),0,J64)</f>
         <v>6</v>
       </c>
       <c r="M64" s="5" t="s">
@@ -12885,9 +13010,13 @@
         <f aca="false">H65*I65</f>
         <v>10</v>
       </c>
-      <c r="K65" s="27"/>
+      <c r="K65" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">O</t>
+        </is>
+      </c>
       <c r="L65" s="26" t="n">
-        <f aca="false">IF(UPPER(K65)="Y",0,J65)</f>
+        <f aca="false">IF(OR(UPPER(K65)="Y",UPPER(K65)="O"),0,J65)</f>
         <v>10</v>
       </c>
       <c r="M65" s="5" t="s">
@@ -12933,9 +13062,13 @@
         <f aca="false">H66*I66</f>
         <v>9</v>
       </c>
-      <c r="K66" s="27"/>
+      <c r="K66" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L66" s="26" t="n">
-        <f aca="false">IF(UPPER(K66)="Y",0,J66)</f>
+        <f aca="false">IF(OR(UPPER(K66)="Y",UPPER(K66)="O"),0,J66)</f>
         <v>9</v>
       </c>
       <c r="M66" s="5" t="s">
@@ -12985,7 +13118,7 @@
       </c>
       <c r="K67" s="27"/>
       <c r="L67" s="26" t="n">
-        <f aca="false">IF(UPPER(K67)="Y",0,J67)</f>
+        <f aca="false">IF(OR(UPPER(K67)="Y",UPPER(K67)="O"),0,J67)</f>
         <v>60</v>
       </c>
       <c r="M67" s="5" t="s">
@@ -13037,7 +13170,7 @@
       </c>
       <c r="K68" s="27"/>
       <c r="L68" s="26" t="n">
-        <f aca="false">IF(UPPER(K68)="Y",0,J68)</f>
+        <f aca="false">IF(OR(UPPER(K68)="Y",UPPER(K68)="O"),0,J68)</f>
         <v>8</v>
       </c>
       <c r="M68" s="5" t="s">
@@ -13087,9 +13220,13 @@
         <f aca="false">H69*I69</f>
         <v>24</v>
       </c>
-      <c r="K69" s="27"/>
+      <c r="K69" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="L69" s="26" t="n">
-        <f aca="false">IF(UPPER(K69)="Y",0,J69)</f>
+        <f aca="false">IF(OR(UPPER(K69)="Y",UPPER(K69)="O"),0,J69)</f>
         <v>24</v>
       </c>
       <c r="M69" s="5" t="s">
@@ -13139,7 +13276,7 @@
         </is>
       </c>
       <c r="L70" s="26" t="n">
-        <f aca="false">IF(UPPER(K70)="Y",0,J70)</f>
+        <f aca="false">IF(OR(UPPER(K70)="Y",UPPER(K70)="O"),0,J70)</f>
         <v>14</v>
       </c>
       <c r="M70" s="5" t="s">
@@ -13191,7 +13328,7 @@
         </is>
       </c>
       <c r="L71" s="26" t="n">
-        <f aca="false">IF(UPPER(K71)="Y",0,J71)</f>
+        <f aca="false">IF(OR(UPPER(K71)="Y",UPPER(K71)="O"),0,J71)</f>
         <v>70</v>
       </c>
       <c r="M71" s="5" t="s">
@@ -13243,7 +13380,7 @@
         </is>
       </c>
       <c r="L72" s="26" t="n">
-        <f aca="false">IF(UPPER(K72)="Y",0,J72)</f>
+        <f aca="false">IF(OR(UPPER(K72)="Y",UPPER(K72)="O"),0,J72)</f>
         <v>18</v>
       </c>
       <c r="M72" s="5" t="s">
@@ -13293,7 +13430,7 @@
         </is>
       </c>
       <c r="L73" s="26" t="n">
-        <f aca="false">IF(UPPER(K73)="Y",0,J73)</f>
+        <f aca="false">IF(OR(UPPER(K73)="Y",UPPER(K73)="O"),0,J73)</f>
         <v>8</v>
       </c>
       <c r="M73" s="5" t="s">
@@ -13343,7 +13480,7 @@
         </is>
       </c>
       <c r="L74" s="26" t="n">
-        <f aca="false">IF(UPPER(K74)="Y",0,J74)</f>
+        <f aca="false">IF(OR(UPPER(K74)="Y",UPPER(K74)="O"),0,J74)</f>
         <v>6</v>
       </c>
       <c r="M74" s="5" t="s">
@@ -13395,7 +13532,7 @@
         </is>
       </c>
       <c r="L75" s="26" t="n">
-        <f aca="false">IF(UPPER(K75)="Y",0,J75)</f>
+        <f aca="false">IF(OR(UPPER(K75)="Y",UPPER(K75)="O"),0,J75)</f>
         <v>6</v>
       </c>
       <c r="M75" s="5" t="s">
@@ -13443,7 +13580,7 @@
       </c>
       <c r="K76" s="27"/>
       <c r="L76" s="26" t="n">
-        <f aca="false">IF(UPPER(K76)="Y",0,J76)</f>
+        <f aca="false">IF(OR(UPPER(K76)="Y",UPPER(K76)="O"),0,J76)</f>
         <v>14</v>
       </c>
       <c r="M76" s="5" t="s">
@@ -13491,7 +13628,7 @@
       </c>
       <c r="K77" s="27"/>
       <c r="L77" s="26" t="n">
-        <f aca="false">IF(UPPER(K77)="Y",0,J77)</f>
+        <f aca="false">IF(OR(UPPER(K77)="Y",UPPER(K77)="O"),0,J77)</f>
         <v>18</v>
       </c>
       <c r="M77" s="5" t="s">
@@ -13543,7 +13680,7 @@
         </is>
       </c>
       <c r="L78" s="26" t="n">
-        <f aca="false">IF(UPPER(K78)="Y",0,J78)</f>
+        <f aca="false">IF(OR(UPPER(K78)="Y",UPPER(K78)="O"),0,J78)</f>
         <v>40</v>
       </c>
       <c r="M78" s="5" t="s">
@@ -13589,7 +13726,7 @@
       </c>
       <c r="K79" s="27"/>
       <c r="L79" s="26" t="n">
-        <f aca="false">IF(UPPER(K79)="Y",0,J79)</f>
+        <f aca="false">IF(OR(UPPER(K79)="Y",UPPER(K79)="O"),0,J79)</f>
         <v>6</v>
       </c>
       <c r="M79" s="5" t="s">
@@ -13635,7 +13772,7 @@
       </c>
       <c r="K80" s="27"/>
       <c r="L80" s="26" t="n">
-        <f aca="false">IF(UPPER(K80)="Y",0,J80)</f>
+        <f aca="false">IF(OR(UPPER(K80)="Y",UPPER(K80)="O"),0,J80)</f>
         <v>22</v>
       </c>
       <c r="M80" s="5" t="s">
@@ -13683,7 +13820,7 @@
       </c>
       <c r="K81" s="27"/>
       <c r="L81" s="26" t="n">
-        <f aca="false">IF(UPPER(K81)="Y",0,J81)</f>
+        <f aca="false">IF(OR(UPPER(K81)="Y",UPPER(K81)="O"),0,J81)</f>
         <v>42</v>
       </c>
       <c r="M81" s="5" t="s">
@@ -13729,7 +13866,7 @@
       </c>
       <c r="K82" s="27"/>
       <c r="L82" s="26" t="n">
-        <f aca="false">IF(UPPER(K82)="Y",0,J82)</f>
+        <f aca="false">IF(OR(UPPER(K82)="Y",UPPER(K82)="O"),0,J82)</f>
         <v>18</v>
       </c>
       <c r="M82" s="5" t="s">
@@ -13777,7 +13914,7 @@
       </c>
       <c r="K83" s="27"/>
       <c r="L83" s="26" t="n">
-        <f aca="false">IF(UPPER(K83)="Y",0,J83)</f>
+        <f aca="false">IF(OR(UPPER(K83)="Y",UPPER(K83)="O"),0,J83)</f>
         <v>69.97</v>
       </c>
       <c r="M83" s="5" t="s">
@@ -13826,7 +13963,7 @@
       </c>
       <c r="K84" s="27"/>
       <c r="L84" s="26" t="n">
-        <f aca="false">IF(UPPER(K84)="Y",0,J84)</f>
+        <f aca="false">IF(OR(UPPER(K84)="Y",UPPER(K84)="O"),0,J84)</f>
         <v>13</v>
       </c>
       <c r="M84" s="5" t="s">
@@ -13875,7 +14012,7 @@
       </c>
       <c r="K85" s="27"/>
       <c r="L85" s="26" t="n">
-        <f aca="false">IF(UPPER(K85)="Y",0,J85)</f>
+        <f aca="false">IF(OR(UPPER(K85)="Y",UPPER(K85)="O"),0,J85)</f>
         <v>12</v>
       </c>
       <c r="M85" s="5" t="s">
@@ -13924,7 +14061,7 @@
       </c>
       <c r="K86" s="27"/>
       <c r="L86" s="26" t="n">
-        <f aca="false">IF(UPPER(K86)="Y",0,J86)</f>
+        <f aca="false">IF(OR(UPPER(K86)="Y",UPPER(K86)="O"),0,J86)</f>
         <v>15</v>
       </c>
       <c r="M86" s="5" t="s">
@@ -13973,7 +14110,7 @@
       </c>
       <c r="K87" s="27"/>
       <c r="L87" s="26" t="n">
-        <f aca="false">IF(UPPER(K87)="Y",0,J87)</f>
+        <f aca="false">IF(OR(UPPER(K87)="Y",UPPER(K87)="O"),0,J87)</f>
         <v>11</v>
       </c>
       <c r="M87" s="5" t="s">
@@ -14022,7 +14159,7 @@
       </c>
       <c r="K88" s="27"/>
       <c r="L88" s="26" t="n">
-        <f aca="false">IF(UPPER(K88)="Y",0,J88)</f>
+        <f aca="false">IF(OR(UPPER(K88)="Y",UPPER(K88)="O"),0,J88)</f>
         <v>6</v>
       </c>
       <c r="M88" s="5" t="s">
@@ -14071,7 +14208,7 @@
       </c>
       <c r="K89" s="27"/>
       <c r="L89" s="26" t="n">
-        <f aca="false">IF(UPPER(K89)="Y",0,J89)</f>
+        <f aca="false">IF(OR(UPPER(K89)="Y",UPPER(K89)="O"),0,J89)</f>
         <v>10</v>
       </c>
       <c r="M89" s="5" t="s">
@@ -14120,7 +14257,7 @@
       </c>
       <c r="K90" s="27"/>
       <c r="L90" s="26" t="n">
-        <f aca="false">IF(UPPER(K90)="Y",0,J90)</f>
+        <f aca="false">IF(OR(UPPER(K90)="Y",UPPER(K90)="O"),0,J90)</f>
         <v>9</v>
       </c>
       <c r="M90" s="5" t="s">
@@ -14167,7 +14304,7 @@
       </c>
       <c r="K91" s="27"/>
       <c r="L91" s="26" t="n">
-        <f aca="false">IF(UPPER(K91)="Y",0,J91)</f>
+        <f aca="false">IF(OR(UPPER(K91)="Y",UPPER(K91)="O"),0,J91)</f>
         <v>7</v>
       </c>
       <c r="M91" s="5" t="s">
@@ -14213,7 +14350,7 @@
       </c>
       <c r="K92" s="27"/>
       <c r="L92" s="26" t="n">
-        <f aca="false">IF(UPPER(K92)="Y",0,J92)</f>
+        <f aca="false">IF(OR(UPPER(K92)="Y",UPPER(K92)="O"),0,J92)</f>
         <v>14</v>
       </c>
       <c r="M92" s="5" t="s">
@@ -14261,7 +14398,7 @@
       </c>
       <c r="K93" s="27"/>
       <c r="L93" s="26" t="n">
-        <f aca="false">IF(UPPER(K93)="Y",0,J93)</f>
+        <f aca="false">IF(OR(UPPER(K93)="Y",UPPER(K93)="O"),0,J93)</f>
         <v>13</v>
       </c>
       <c r="M93" s="5" t="s">
@@ -14309,7 +14446,7 @@
       </c>
       <c r="K94" s="27"/>
       <c r="L94" s="26" t="n">
-        <f aca="false">IF(UPPER(K94)="Y",0,J94)</f>
+        <f aca="false">IF(OR(UPPER(K94)="Y",UPPER(K94)="O"),0,J94)</f>
         <v>12</v>
       </c>
       <c r="M94" s="5" t="s">
@@ -14355,7 +14492,7 @@
       </c>
       <c r="K95" s="27"/>
       <c r="L95" s="26" t="n">
-        <f aca="false">IF(UPPER(K95)="Y",0,J95)</f>
+        <f aca="false">IF(OR(UPPER(K95)="Y",UPPER(K95)="O"),0,J95)</f>
         <v>8</v>
       </c>
       <c r="M95" s="5" t="s">
@@ -14401,7 +14538,7 @@
       </c>
       <c r="K96" s="27"/>
       <c r="L96" s="26" t="n">
-        <f aca="false">IF(UPPER(K96)="Y",0,J96)</f>
+        <f aca="false">IF(OR(UPPER(K96)="Y",UPPER(K96)="O"),0,J96)</f>
         <v>6</v>
       </c>
       <c r="M96" s="5" t="s">
@@ -14449,7 +14586,7 @@
       </c>
       <c r="K97" s="27"/>
       <c r="L97" s="26" t="n">
-        <f aca="false">IF(UPPER(K97)="Y",0,J97)</f>
+        <f aca="false">IF(OR(UPPER(K97)="Y",UPPER(K97)="O"),0,J97)</f>
         <v>5</v>
       </c>
       <c r="M97" s="5" t="s">
@@ -14495,7 +14632,7 @@
       </c>
       <c r="K98" s="27"/>
       <c r="L98" s="26" t="n">
-        <f aca="false">IF(UPPER(K98)="Y",0,J98)</f>
+        <f aca="false">IF(OR(UPPER(K98)="Y",UPPER(K98)="O"),0,J98)</f>
         <v>6</v>
       </c>
       <c r="M98" s="5" t="s">
@@ -14541,7 +14678,7 @@
       </c>
       <c r="K99" s="27"/>
       <c r="L99" s="26" t="n">
-        <f aca="false">IF(UPPER(K99)="Y",0,J99)</f>
+        <f aca="false">IF(OR(UPPER(K99)="Y",UPPER(K99)="O"),0,J99)</f>
         <v>8</v>
       </c>
       <c r="M99" s="5" t="s">
@@ -14585,7 +14722,7 @@
       </c>
       <c r="K100" s="27"/>
       <c r="L100" s="26" t="n">
-        <f aca="false">IF(UPPER(K100)="Y",0,J100)</f>
+        <f aca="false">IF(OR(UPPER(K100)="Y",UPPER(K100)="O"),0,J100)</f>
         <v>9</v>
       </c>
       <c r="M100" s="5" t="s">
@@ -14633,7 +14770,7 @@
       </c>
       <c r="K101" s="27"/>
       <c r="L101" s="26" t="n">
-        <f aca="false">IF(UPPER(K101)="Y",0,J101)</f>
+        <f aca="false">IF(OR(UPPER(K101)="Y",UPPER(K101)="O"),0,J101)</f>
         <v>8</v>
       </c>
       <c r="M101" s="5" t="s">
@@ -14679,7 +14816,7 @@
       </c>
       <c r="K102" s="27"/>
       <c r="L102" s="26" t="n">
-        <f aca="false">IF(UPPER(K102)="Y",0,J102)</f>
+        <f aca="false">IF(OR(UPPER(K102)="Y",UPPER(K102)="O"),0,J102)</f>
         <v>6</v>
       </c>
       <c r="M102" s="5" t="s">
@@ -14727,7 +14864,7 @@
       </c>
       <c r="K103" s="27"/>
       <c r="L103" s="26" t="n">
-        <f aca="false">IF(UPPER(K103)="Y",0,J103)</f>
+        <f aca="false">IF(OR(UPPER(K103)="Y",UPPER(K103)="O"),0,J103)</f>
         <v>9</v>
       </c>
       <c r="M103" s="5" t="s">
@@ -14773,7 +14910,7 @@
       </c>
       <c r="K104" s="27"/>
       <c r="L104" s="26" t="n">
-        <f aca="false">IF(UPPER(K104)="Y",0,J104)</f>
+        <f aca="false">IF(OR(UPPER(K104)="Y",UPPER(K104)="O"),0,J104)</f>
         <v>7</v>
       </c>
       <c r="M104" s="5" t="s">
@@ -14819,7 +14956,7 @@
       </c>
       <c r="K105" s="27"/>
       <c r="L105" s="26" t="n">
-        <f aca="false">IF(UPPER(K105)="Y",0,J105)</f>
+        <f aca="false">IF(OR(UPPER(K105)="Y",UPPER(K105)="O"),0,J105)</f>
         <v>7</v>
       </c>
       <c r="M105" s="5" t="s">
@@ -14865,7 +15002,7 @@
       </c>
       <c r="K106" s="27"/>
       <c r="L106" s="26" t="n">
-        <f aca="false">IF(UPPER(K106)="Y",0,J106)</f>
+        <f aca="false">IF(OR(UPPER(K106)="Y",UPPER(K106)="O"),0,J106)</f>
         <v>13</v>
       </c>
       <c r="M106" s="5" t="s">
@@ -14914,7 +15051,7 @@
       </c>
       <c r="K107" s="27"/>
       <c r="L107" s="26" t="n">
-        <f aca="false">IF(UPPER(K107)="Y",0,J107)</f>
+        <f aca="false">IF(OR(UPPER(K107)="Y",UPPER(K107)="O"),0,J107)</f>
         <v>20</v>
       </c>
       <c r="M107" s="5" t="s">
@@ -14963,7 +15100,7 @@
       </c>
       <c r="K108" s="27"/>
       <c r="L108" s="26" t="n">
-        <f aca="false">IF(UPPER(K108)="Y",0,J108)</f>
+        <f aca="false">IF(OR(UPPER(K108)="Y",UPPER(K108)="O"),0,J108)</f>
         <v>24</v>
       </c>
       <c r="M108" s="5" t="s">
@@ -15011,7 +15148,7 @@
       </c>
       <c r="K109" s="27"/>
       <c r="L109" s="26" t="n">
-        <f aca="false">IF(UPPER(K109)="Y",0,J109)</f>
+        <f aca="false">IF(OR(UPPER(K109)="Y",UPPER(K109)="O"),0,J109)</f>
         <v>18</v>
       </c>
       <c r="M109" s="5" t="s">
@@ -15041,7 +15178,7 @@
   <autoFilter ref="A1:O109"/>
   <dataValidations count="1">
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="K2:K109" type="list">
-      <formula1>"Y,N"</formula1>
+      <formula1>"Y,O,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -15120,7 +15257,11 @@
       <c r="C3" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="D3" s="27"/>
+      <c r="D3" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E3" s="9" t="n">
         <f aca="false">IF(UPPER(D3)="Y",0,C3)</f>
         <v>8</v>
@@ -15156,7 +15297,11 @@
       <c r="C5" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="D5" s="27"/>
+      <c r="D5" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E5" s="9" t="n">
         <f aca="false">IF(UPPER(D5)="Y",0,C5)</f>
         <v>12</v>
@@ -15173,7 +15318,11 @@
       <c r="C6" s="30" t="n">
         <v>18</v>
       </c>
-      <c r="D6" s="27"/>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E6" s="9" t="n">
         <f aca="false">IF(UPPER(D6)="Y",0,C6)</f>
         <v>18</v>
@@ -15300,7 +15449,11 @@
       <c r="C13" s="30" t="n">
         <v>12</v>
       </c>
-      <c r="D13" s="27"/>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E13" s="9" t="n">
         <f aca="false">IF(UPPER(D13)="Y",0,C13)</f>
         <v>12</v>
@@ -15378,7 +15531,11 @@
       <c r="C17" s="30" t="n">
         <v>15</v>
       </c>
-      <c r="D17" s="27"/>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="E17" s="9" t="n">
         <f aca="false">IF(UPPER(D17)="Y",0,C17)</f>
         <v>15</v>

</xml_diff>